<commit_message>
Added AU sweeping of pop out method.
</commit_message>
<xml_diff>
--- a/results/02_taxa_assemblage/LDA_Method/ModelFinalized/tables/anova/anova_env.xlsx
+++ b/results/02_taxa_assemblage/LDA_Method/ModelFinalized/tables/anova/anova_env.xlsx
@@ -490,19 +490,19 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>77.62</v>
+        <v>94.23</v>
       </c>
       <c r="D2" t="n">
         <v>2</v>
       </c>
       <c r="E2" t="n">
-        <v>136.74</v>
+        <v>120.13</v>
       </c>
       <c r="F2" t="n">
         <v>307</v>
       </c>
       <c r="G2" t="n">
-        <v>87.13</v>
+        <v>120.4</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -511,17 +511,17 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>1.47 ± 0.04</t>
+          <t>1.42 ± 0.04</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>1.53 ± 0.13</t>
+          <t>1.23 ± 0.23</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>0.38 ± 0.09</t>
+          <t>-0.03 ± 0.10</t>
         </is>
       </c>
     </row>
@@ -535,19 +535,19 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>223.24</v>
+        <v>66.59999999999999</v>
       </c>
       <c r="D3" t="n">
         <v>2</v>
       </c>
       <c r="E3" t="n">
-        <v>516.08</v>
+        <v>672.71</v>
       </c>
       <c r="F3" t="n">
         <v>307</v>
       </c>
       <c r="G3" t="n">
-        <v>66.40000000000001</v>
+        <v>15.2</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -556,17 +556,17 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>9.39 ± 0.08</t>
+          <t>9.17 ± 0.09</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>10.20 ± 0.39</t>
+          <t>9.31 ± 0.33</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>7.70 ± 0.14</t>
+          <t>7.97 ± 0.21</t>
         </is>
       </c>
     </row>
@@ -576,23 +576,23 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Measured Depth (m)</t>
+          <t>LOI (%)</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>573.8200000000001</v>
+        <v>122.5</v>
       </c>
       <c r="D4" t="n">
         <v>2</v>
       </c>
       <c r="E4" t="n">
-        <v>2384.81</v>
+        <v>1682.66</v>
       </c>
       <c r="F4" t="n">
         <v>307</v>
       </c>
       <c r="G4" t="n">
-        <v>36.93</v>
+        <v>11.17</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -601,17 +601,17 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>3.08 ± 0.17</t>
+          <t>2.88 ± 0.13</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>6.88 ± 0.69</t>
+          <t>1.21 ± 0.14</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>5.42 ± 0.35</t>
+          <t>4.22 ± 0.48</t>
         </is>
       </c>
     </row>
@@ -621,23 +621,23 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>LOI (%)</t>
+          <t>Measured Depth (m)</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>113.83</v>
+        <v>186.35</v>
       </c>
       <c r="D5" t="n">
         <v>2</v>
       </c>
       <c r="E5" t="n">
-        <v>1691.33</v>
+        <v>2772.27</v>
       </c>
       <c r="F5" t="n">
         <v>307</v>
       </c>
       <c r="G5" t="n">
-        <v>10.33</v>
+        <v>10.32</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -646,17 +646,17 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2.74 ± 0.13</t>
+          <t>3.79 ± 0.19</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2.24 ± 0.34</t>
+          <t>3.03 ± 0.49</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>3.97 ± 0.34</t>
+          <t>5.75 ± 0.44</t>
         </is>
       </c>
     </row>
@@ -670,38 +670,38 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>40.41</v>
+        <v>72.25</v>
       </c>
       <c r="D6" t="n">
         <v>2</v>
       </c>
       <c r="E6" t="n">
-        <v>1815.39</v>
+        <v>1783.55</v>
       </c>
       <c r="F6" t="n">
         <v>307</v>
       </c>
       <c r="G6" t="n">
-        <v>3.42</v>
+        <v>6.22</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>0.0341*</t>
+          <t>0.0023**</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>19.53 ± 0.17</t>
+          <t>19.56 ± 0.16</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>19.62 ± 0.64</t>
+          <t>21.76 ± 0.61</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>20.33 ± 0.23</t>
+          <t>20.28 ± 0.28</t>
         </is>
       </c>
     </row>
@@ -736,13 +736,13 @@
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="n">
-        <v>191</v>
+        <v>243</v>
       </c>
       <c r="J8" t="n">
-        <v>28</v>
+        <v>12</v>
       </c>
       <c r="K8" t="n">
-        <v>91</v>
+        <v>55</v>
       </c>
     </row>
     <row r="9">

</xml_diff>